<commit_message>
29 NOV 2025 CLOSING
</commit_message>
<xml_diff>
--- a/SUPPLIER RELATED/SUPPLIER PAYMENT STATUS.xlsx
+++ b/SUPPLIER RELATED/SUPPLIER PAYMENT STATUS.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16040"/>
+    <workbookView windowWidth="19635" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="SUPPLIER PAYMENT STATUS" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="70">
   <si>
     <t>DIVISION</t>
   </si>
@@ -65,15 +65,15 @@
     <t>SEDANA JAYA</t>
   </si>
   <si>
+    <t>Sedana</t>
+  </si>
+  <si>
+    <t>RAFI SEAFOOD</t>
+  </si>
+  <si>
     <t>POSTED</t>
   </si>
   <si>
-    <t>Sedana</t>
-  </si>
-  <si>
-    <t>RAFI SEAFOOD</t>
-  </si>
-  <si>
     <t>Surbled</t>
   </si>
   <si>
@@ -159,9 +159,6 @@
   </si>
   <si>
     <t>NANO DEWATA</t>
-  </si>
-  <si>
-    <t>UNCHECKED</t>
   </si>
   <si>
     <t>BALI PERMATA JAYA</t>
@@ -247,12 +244,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="6">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="180" formatCode="[$-409]d\-mmm\-yyyy;@"/>
-    <numFmt numFmtId="181" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -428,7 +425,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,12 +470,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -664,7 +655,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -712,6 +703,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -729,6 +735,21 @@
         <color auto="1"/>
       </left>
       <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
         <color auto="1"/>
       </right>
       <top style="thin">
@@ -782,7 +803,35 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
         <color auto="1"/>
       </right>
       <top/>
@@ -822,7 +871,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color auto="1"/>
       </left>
       <right style="thin">
@@ -831,7 +880,9 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -856,77 +907,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1035,16 +1015,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1053,7 +1033,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1065,115 +1045,115 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1181,7 +1161,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1190,10 +1170,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1202,40 +1182,58 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1244,28 +1242,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1274,52 +1257,49 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1856,20 +1836,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L53"/>
-  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9.16190476190476" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="18.859375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="33.3359375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.3359375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.3359375" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" style="3" customWidth="1"/>
-    <col min="6" max="7" width="13.6640625" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="14.3359375"/>
-    <col min="10" max="10" width="15.4296875"/>
-    <col min="11" max="11" width="14.3359375"/>
-    <col min="12" max="12" width="22.6640625" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625"/>
+    <col min="1" max="1" width="18.8571428571429" style="1" customWidth="1"/>
+    <col min="2" max="2" width="33.3333333333333" style="2" customWidth="1"/>
+    <col min="3" max="3" width="14.3333333333333" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.3333333333333" customWidth="1"/>
+    <col min="5" max="5" width="12.5714285714286" style="3" customWidth="1"/>
+    <col min="6" max="7" width="13.6666666666667" customWidth="1"/>
+    <col min="8" max="8" width="13.6666666666667" style="4" customWidth="1"/>
+    <col min="9" max="9" width="14.3333333333333"/>
+    <col min="10" max="10" width="15.4285714285714"/>
+    <col min="11" max="11" width="14.3333333333333"/>
+    <col min="12" max="12" width="22.6666666666667" customWidth="1"/>
+    <col min="13" max="13" width="11.6666666666667"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1885,886 +1865,886 @@
       <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="39" t="s">
+      <c r="G1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="J1" s="47">
-        <f>SUM(F2,F3,F4,F8,F13,F14,F17,F24,F25,F34,F46)</f>
-        <v>129392646</v>
-      </c>
-    </row>
-    <row r="2" ht="16.8" spans="1:10">
-      <c r="A2" s="9" t="s">
+        <f>SUM(F2,F4,F8,F13,F14,F17,F24,F25,F34)</f>
+        <v>88565236</v>
+      </c>
+    </row>
+    <row r="2" ht="15" spans="1:10">
+      <c r="A2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="12">
+      <c r="C2" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="15">
         <v>66835000</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="15">
         <v>39738000</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="41"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="16"/>
       <c r="J2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="16.8" spans="1:10">
-      <c r="A3" s="13"/>
-      <c r="B3" s="10" t="s">
+    <row r="3" ht="15" spans="1:10">
+      <c r="A3" s="17"/>
+      <c r="B3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="12">
+      <c r="C3" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="15">
         <v>45478060</v>
       </c>
-      <c r="E3" s="34" t="s">
+      <c r="E3" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="15">
+        <v>39027410</v>
+      </c>
+      <c r="G3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="J3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="12">
-        <v>39027410</v>
-      </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="41"/>
-      <c r="J3" t="s">
+    </row>
+    <row r="4" ht="15" spans="1:10">
+      <c r="A4" s="17"/>
+      <c r="B4" s="13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" ht="16.8" spans="1:10">
-      <c r="A4" s="13"/>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="15">
+        <v>29900100</v>
+      </c>
+      <c r="E4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="12">
-        <v>29900100</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="12">
+      <c r="F4" s="15">
         <v>20617200</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="41"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="16"/>
       <c r="J4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" ht="16.8" spans="1:10">
-      <c r="A5" s="13"/>
-      <c r="B5" s="10" t="s">
+    <row r="5" ht="15" spans="1:10">
+      <c r="A5" s="17"/>
+      <c r="B5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="12">
+      <c r="C5" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="15">
         <v>4400000</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="12">
+      <c r="E5" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="15">
         <v>5560000</v>
       </c>
-      <c r="G5" s="12"/>
-      <c r="H5" s="41"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="16"/>
       <c r="J5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" ht="16.8" spans="1:10">
-      <c r="A6" s="13"/>
-      <c r="B6" s="10" t="s">
+    <row r="6" ht="15" spans="1:10">
+      <c r="A6" s="17"/>
+      <c r="B6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="12">
+      <c r="C6" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="15">
         <v>5610900</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="12">
+      <c r="E6" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="15">
         <v>3578050</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="41"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="16"/>
       <c r="J6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" ht="16.8" spans="1:10">
-      <c r="A7" s="13"/>
-      <c r="B7" s="10" t="s">
+    <row r="7" ht="15" spans="1:10">
+      <c r="A7" s="17"/>
+      <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="12">
+      <c r="C7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="15">
         <v>3663300</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="12">
+      <c r="E7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="15">
         <v>1983600</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="41"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="16"/>
       <c r="J7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" ht="16.8" spans="1:10">
-      <c r="A8" s="13"/>
-      <c r="B8" s="10" t="s">
+    <row r="8" ht="15" spans="1:10">
+      <c r="A8" s="17"/>
+      <c r="B8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="12">
+      <c r="C8" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="15">
         <v>8775000</v>
       </c>
-      <c r="E8" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="12">
+      <c r="E8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="15">
         <v>7800000</v>
       </c>
-      <c r="G8" s="12"/>
-      <c r="H8" s="41"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="16"/>
       <c r="J8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" ht="16.8" spans="1:8">
-      <c r="A9" s="13"/>
-      <c r="B9" s="10" t="s">
+    <row r="9" ht="15" spans="1:8">
+      <c r="A9" s="17"/>
+      <c r="B9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="14" t="s">
+      <c r="D9" s="15"/>
+      <c r="E9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="41"/>
-    </row>
-    <row r="10" ht="16.8" spans="1:10">
-      <c r="A10" s="13"/>
-      <c r="B10" s="10" t="s">
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
+    </row>
+    <row r="10" ht="15" spans="1:10">
+      <c r="A10" s="17"/>
+      <c r="B10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="14" t="s">
+      <c r="D10" s="15"/>
+      <c r="E10" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="41"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="16"/>
       <c r="J10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" ht="16.8" spans="1:12">
-      <c r="A11" s="13"/>
-      <c r="B11" s="10" t="s">
+    <row r="11" ht="15" spans="1:12">
+      <c r="A11" s="17"/>
+      <c r="B11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="12">
+      <c r="D11" s="15"/>
+      <c r="E11" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="15">
         <v>326000</v>
       </c>
-      <c r="G11" s="12"/>
-      <c r="H11" s="41"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="16"/>
       <c r="J11" t="s">
         <v>29</v>
       </c>
       <c r="L11" s="47"/>
     </row>
-    <row r="12" ht="16.8" spans="1:10">
-      <c r="A12" s="13"/>
-      <c r="B12" s="10" t="s">
+    <row r="12" ht="15" spans="1:10">
+      <c r="A12" s="17"/>
+      <c r="B12" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="12">
+      <c r="C12" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="15">
         <v>924000</v>
       </c>
-      <c r="G12" s="12"/>
-      <c r="H12" s="41"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="16"/>
       <c r="J12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" ht="16.8" spans="1:10">
-      <c r="A13" s="13"/>
-      <c r="B13" s="10" t="s">
+    <row r="13" ht="15" spans="1:10">
+      <c r="A13" s="17"/>
+      <c r="B13" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="12">
+      <c r="C13" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="15">
         <v>4375000</v>
       </c>
-      <c r="E13" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="12">
+      <c r="E13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="15">
         <v>4715000</v>
       </c>
-      <c r="G13" s="12"/>
-      <c r="H13" s="41"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="16"/>
       <c r="J13" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" ht="16.8" spans="1:8">
-      <c r="A14" s="13"/>
-      <c r="B14" s="10" t="s">
+    <row r="14" ht="15" spans="1:8">
+      <c r="A14" s="17"/>
+      <c r="B14" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="12">
+      <c r="C14" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="15">
         <v>1525000</v>
       </c>
-      <c r="G14" s="12"/>
-      <c r="H14" s="41"/>
-    </row>
-    <row r="15" ht="17.55" spans="1:8">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16" t="s">
+      <c r="G14" s="15"/>
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="20"/>
+      <c r="B15" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="18">
+      <c r="C15" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="23"/>
+      <c r="E15" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="23">
         <v>2320000</v>
       </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="42"/>
-    </row>
-    <row r="16" ht="16.8" spans="1:8">
-      <c r="A16" s="19" t="s">
+      <c r="G15" s="23"/>
+      <c r="H15" s="24"/>
+    </row>
+    <row r="16" ht="15" spans="1:8">
+      <c r="A16" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="22">
+      <c r="C16" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="28">
         <v>20669000</v>
       </c>
-      <c r="E16" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="22">
+      <c r="E16" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="28">
         <v>13909500</v>
       </c>
-      <c r="G16" s="22"/>
-      <c r="H16" s="43"/>
-    </row>
-    <row r="17" ht="16.8" spans="1:8">
-      <c r="A17" s="13"/>
-      <c r="B17" s="10" t="s">
+      <c r="G16" s="28"/>
+      <c r="H16" s="29"/>
+    </row>
+    <row r="17" ht="15" spans="1:8">
+      <c r="A17" s="17"/>
+      <c r="B17" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="12">
+      <c r="C17" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="15">
         <v>3230000</v>
       </c>
-      <c r="E17" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="12">
+      <c r="E17" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="15">
         <v>2415000</v>
       </c>
-      <c r="G17" s="12"/>
-      <c r="H17" s="41"/>
-    </row>
-    <row r="18" ht="16.8" spans="1:8">
-      <c r="A18" s="13"/>
-      <c r="B18" s="10" t="s">
+      <c r="G17" s="15"/>
+      <c r="H17" s="16"/>
+    </row>
+    <row r="18" ht="15" spans="1:8">
+      <c r="A18" s="17"/>
+      <c r="B18" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="12">
+      <c r="C18" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="15">
         <v>10775000</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="12">
+      <c r="E18" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="15">
         <v>10000000</v>
       </c>
-      <c r="G18" s="12"/>
-      <c r="H18" s="41"/>
-    </row>
-    <row r="19" ht="16.8" spans="1:8">
-      <c r="A19" s="13"/>
-      <c r="B19" s="10" t="s">
+      <c r="G18" s="15"/>
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" ht="15" spans="1:8">
+      <c r="A19" s="17"/>
+      <c r="B19" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="12">
+      <c r="C19" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="15">
         <v>10023000</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="12">
+      <c r="E19" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="15">
         <v>6637500</v>
       </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="41"/>
-    </row>
-    <row r="20" ht="16.8" spans="1:8">
-      <c r="A20" s="13"/>
-      <c r="B20" s="10" t="s">
+      <c r="G19" s="15"/>
+      <c r="H19" s="16"/>
+    </row>
+    <row r="20" ht="15" spans="1:8">
+      <c r="A20" s="17"/>
+      <c r="B20" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="14" t="s">
+      <c r="D20" s="15"/>
+      <c r="E20" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="41"/>
-    </row>
-    <row r="21" ht="16.8" spans="1:8">
-      <c r="A21" s="13"/>
-      <c r="B21" s="10" t="s">
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="16"/>
+    </row>
+    <row r="21" ht="15" spans="1:8">
+      <c r="A21" s="17"/>
+      <c r="B21" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="12">
+      <c r="C21" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="15">
         <v>3663000</v>
       </c>
-      <c r="E21" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="12">
+      <c r="E21" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="15">
         <v>1998000</v>
       </c>
-      <c r="G21" s="12"/>
-      <c r="H21" s="41"/>
-    </row>
-    <row r="22" ht="16.8" spans="1:8">
-      <c r="A22" s="13"/>
-      <c r="B22" s="10" t="s">
+      <c r="G21" s="15"/>
+      <c r="H21" s="16"/>
+    </row>
+    <row r="22" ht="15" spans="1:8">
+      <c r="A22" s="17"/>
+      <c r="B22" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="12">
+      <c r="C22" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="15">
         <v>2410000</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="41"/>
-    </row>
-    <row r="23" ht="16.8" spans="1:8">
-      <c r="A23" s="13"/>
-      <c r="B23" s="10" t="s">
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="16"/>
+    </row>
+    <row r="23" ht="15" spans="1:8">
+      <c r="A23" s="17"/>
+      <c r="B23" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="12">
+      <c r="C23" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="15">
         <v>2447502</v>
       </c>
-      <c r="E23" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="12">
+      <c r="E23" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="15">
         <v>1312502</v>
       </c>
-      <c r="G23" s="12"/>
-      <c r="H23" s="41"/>
-    </row>
-    <row r="24" ht="16.8" spans="1:8">
-      <c r="A24" s="13"/>
-      <c r="B24" s="10" t="s">
+      <c r="G23" s="15"/>
+      <c r="H23" s="16"/>
+    </row>
+    <row r="24" ht="15" spans="1:8">
+      <c r="A24" s="17"/>
+      <c r="B24" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" s="15"/>
+      <c r="E24" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="15">
+        <v>2280000</v>
+      </c>
+      <c r="G24" s="15"/>
+      <c r="H24" s="16"/>
+    </row>
+    <row r="25" ht="15" spans="1:8">
+      <c r="A25" s="17"/>
+      <c r="B25" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="12">
-        <v>2280000</v>
-      </c>
-      <c r="G24" s="12"/>
-      <c r="H24" s="41"/>
-    </row>
-    <row r="25" ht="16.8" spans="1:8">
-      <c r="A25" s="13"/>
-      <c r="B25" s="10" t="s">
+      <c r="C25" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="15">
+        <v>4760036</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="15">
+        <v>4760036</v>
+      </c>
+      <c r="G25" s="15"/>
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" ht="15" spans="1:8">
+      <c r="A26" s="17"/>
+      <c r="B26" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="12">
-        <v>4760036</v>
-      </c>
-      <c r="E25" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F25" s="12">
-        <v>4760036</v>
-      </c>
-      <c r="G25" s="12"/>
-      <c r="H25" s="41"/>
-    </row>
-    <row r="26" ht="16.8" spans="1:8">
-      <c r="A26" s="13"/>
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="15">
+        <v>5600000</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="15">
+        <v>5600000</v>
+      </c>
+      <c r="G26" s="15"/>
+      <c r="H26" s="16"/>
+    </row>
+    <row r="27" ht="15" spans="1:8">
+      <c r="A27" s="17"/>
+      <c r="B27" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="12">
-        <v>5600000</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="12">
-        <v>5600000</v>
-      </c>
-      <c r="G26" s="12"/>
-      <c r="H26" s="41"/>
-    </row>
-    <row r="27" ht="16.8" spans="1:8">
-      <c r="A27" s="13"/>
-      <c r="B27" s="10" t="s">
+      <c r="C27" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="15">
+        <v>1225000</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="15">
+        <v>915750</v>
+      </c>
+      <c r="G27" s="15"/>
+      <c r="H27" s="16"/>
+    </row>
+    <row r="28" ht="15" spans="1:8">
+      <c r="A28" s="17"/>
+      <c r="B28" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="12">
-        <v>1225000</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" s="12">
+      <c r="C28" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="16"/>
+    </row>
+    <row r="29" ht="15" spans="1:8">
+      <c r="A29" s="17"/>
+      <c r="B29" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="15">
+        <v>3948000</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="16"/>
+    </row>
+    <row r="30" ht="15" spans="1:8">
+      <c r="A30" s="17"/>
+      <c r="B30" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="15">
+        <v>250000</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="16"/>
+    </row>
+    <row r="31" ht="15" spans="1:8">
+      <c r="A31" s="17"/>
+      <c r="B31" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="16"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="20"/>
+      <c r="B32" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="33"/>
+      <c r="E32" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="33">
         <v>915750</v>
       </c>
-      <c r="G27" s="12"/>
-      <c r="H27" s="41"/>
-    </row>
-    <row r="28" ht="16.8" spans="1:8">
-      <c r="A28" s="13"/>
-      <c r="B28" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="41"/>
-    </row>
-    <row r="29" ht="16.8" spans="1:8">
-      <c r="A29" s="13"/>
-      <c r="B29" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="12">
-        <v>3948000</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="41"/>
-    </row>
-    <row r="30" ht="16.8" spans="1:8">
-      <c r="A30" s="13"/>
-      <c r="B30" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="12">
-        <v>250000</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="41"/>
-    </row>
-    <row r="31" ht="16.8" spans="1:8">
-      <c r="A31" s="13"/>
-      <c r="B31" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C31" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="41"/>
-    </row>
-    <row r="32" ht="17.55" spans="1:8">
-      <c r="A32" s="15"/>
-      <c r="B32" s="25" t="s">
+      <c r="G32" s="33"/>
+      <c r="H32" s="34"/>
+    </row>
+    <row r="33" ht="15" spans="1:8">
+      <c r="A33" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="F32" s="27">
-        <v>915750</v>
-      </c>
-      <c r="G32" s="27"/>
-      <c r="H32" s="44"/>
-    </row>
-    <row r="33" ht="16.8" spans="1:8">
-      <c r="A33" s="28" t="s">
+      <c r="B33" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="C33" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="28">
+        <v>4897000</v>
+      </c>
+      <c r="E33" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="28">
+        <v>8368100</v>
+      </c>
+      <c r="G33" s="28"/>
+      <c r="H33" s="29"/>
+    </row>
+    <row r="34" ht="15" spans="1:8">
+      <c r="A34" s="36"/>
+      <c r="B34" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C33" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="22">
-        <v>4897000</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="F33" s="22">
-        <v>8368100</v>
-      </c>
-      <c r="G33" s="22"/>
-      <c r="H33" s="43"/>
-    </row>
-    <row r="34" ht="16.8" spans="1:8">
-      <c r="A34" s="29"/>
-      <c r="B34" s="10" t="s">
+      <c r="C34" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="15">
+        <v>4375000</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" s="15">
+        <v>4715000</v>
+      </c>
+      <c r="G34" s="15"/>
+      <c r="H34" s="16"/>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="36"/>
+      <c r="B35" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="12">
-        <v>4375000</v>
-      </c>
-      <c r="E34" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="12">
-        <v>4715000</v>
-      </c>
-      <c r="G34" s="12"/>
-      <c r="H34" s="41"/>
-    </row>
-    <row r="35" ht="16.8" spans="1:8">
-      <c r="A35" s="29"/>
-      <c r="B35" s="10" t="s">
+      <c r="C35" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="15">
+        <v>1007480.64</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="15">
+        <v>638483</v>
+      </c>
+      <c r="G35" s="15"/>
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="38"/>
+      <c r="B36" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="12">
-        <v>1007480.64</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F35" s="12">
-        <v>638483</v>
-      </c>
-      <c r="G35" s="12"/>
-      <c r="H35" s="41"/>
-    </row>
-    <row r="36" ht="16.8" spans="1:8">
-      <c r="A36" s="9"/>
-      <c r="B36" s="30" t="s">
+      <c r="C36" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="23">
+        <v>1168000</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="23">
+        <v>893000</v>
+      </c>
+      <c r="G36" s="23"/>
+      <c r="H36" s="24"/>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="C36" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="32">
-        <v>1168000</v>
-      </c>
-      <c r="E36" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="F36" s="32">
-        <v>893000</v>
-      </c>
-      <c r="G36" s="32"/>
-      <c r="H36" s="46"/>
-    </row>
-    <row r="37" ht="16.8" spans="1:8">
-      <c r="A37" s="33" t="s">
+      <c r="B37" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="C37" s="41"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" s="44">
+        <v>1020000</v>
+      </c>
+      <c r="G37" s="42"/>
+      <c r="H37" s="44"/>
+    </row>
+    <row r="38" ht="15" spans="1:8">
+      <c r="A38" s="39"/>
+      <c r="B38" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="34"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" s="12">
-        <v>1020000</v>
-      </c>
-      <c r="G37" s="35"/>
-      <c r="H37" s="12"/>
-    </row>
-    <row r="38" ht="16.8" spans="1:8">
-      <c r="A38" s="36"/>
-      <c r="B38" s="10" t="s">
+      <c r="C38" s="18"/>
+      <c r="D38" s="45"/>
+      <c r="E38" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="G38" s="45"/>
+      <c r="H38" s="15"/>
+    </row>
+    <row r="39" ht="15" spans="1:8">
+      <c r="A39" s="39"/>
+      <c r="B39" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C38" s="34"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F38" s="12">
-        <v>1350000</v>
-      </c>
-      <c r="G38" s="35"/>
-      <c r="H38" s="12"/>
-    </row>
-    <row r="39" ht="16.8" spans="1:8">
-      <c r="A39" s="36"/>
-      <c r="B39" s="10" t="s">
+      <c r="C39" s="18"/>
+      <c r="D39" s="45"/>
+      <c r="E39" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="15">
+        <v>600000</v>
+      </c>
+      <c r="G39" s="45"/>
+      <c r="H39" s="15"/>
+    </row>
+    <row r="40" ht="15" spans="1:8">
+      <c r="A40" s="39"/>
+      <c r="B40" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C39" s="34"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F39" s="12">
-        <v>600000</v>
-      </c>
-      <c r="G39" s="35"/>
-      <c r="H39" s="12"/>
-    </row>
-    <row r="40" ht="16.8" spans="1:8">
-      <c r="A40" s="36"/>
-      <c r="B40" s="10" t="s">
+      <c r="C40" s="18"/>
+      <c r="D40" s="45"/>
+      <c r="E40" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" s="15">
+        <v>318134</v>
+      </c>
+      <c r="G40" s="45"/>
+      <c r="H40" s="15"/>
+    </row>
+    <row r="41" ht="15" spans="1:8">
+      <c r="A41" s="39"/>
+      <c r="B41" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="34"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F40" s="12">
-        <v>318134</v>
-      </c>
-      <c r="G40" s="35"/>
-      <c r="H40" s="12"/>
-    </row>
-    <row r="41" ht="16.8" spans="1:8">
-      <c r="A41" s="36"/>
-      <c r="B41" s="10" t="s">
+      <c r="C41" s="18"/>
+      <c r="D41" s="45"/>
+      <c r="E41" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" s="15">
+        <v>248700</v>
+      </c>
+      <c r="G41" s="45"/>
+      <c r="H41" s="15"/>
+    </row>
+    <row r="42" ht="15" spans="1:8">
+      <c r="A42" s="39"/>
+      <c r="B42" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C41" s="34"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F41" s="12">
-        <v>248700</v>
-      </c>
-      <c r="G41" s="35"/>
-      <c r="H41" s="12"/>
-    </row>
-    <row r="42" ht="16.8" spans="1:8">
-      <c r="A42" s="36"/>
-      <c r="B42" s="10" t="s">
+      <c r="C42" s="18"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F42" s="15">
+        <v>1029180</v>
+      </c>
+      <c r="G42" s="45"/>
+      <c r="H42" s="15"/>
+    </row>
+    <row r="43" ht="15" spans="1:8">
+      <c r="A43" s="39"/>
+      <c r="B43" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="34"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F42" s="12">
-        <v>1029180</v>
-      </c>
-      <c r="G42" s="35"/>
-      <c r="H42" s="12"/>
-    </row>
-    <row r="43" ht="16.8" spans="1:8">
-      <c r="A43" s="36"/>
-      <c r="B43" s="10" t="s">
+      <c r="C43" s="18"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F43" s="15">
+        <v>270000</v>
+      </c>
+      <c r="G43" s="45"/>
+      <c r="H43" s="15"/>
+    </row>
+    <row r="44" ht="15" spans="1:8">
+      <c r="A44" s="39"/>
+      <c r="B44" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C43" s="34"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F43" s="12">
-        <v>270000</v>
-      </c>
-      <c r="G43" s="35"/>
-      <c r="H43" s="12"/>
-    </row>
-    <row r="44" ht="16.8" spans="1:8">
-      <c r="A44" s="36"/>
-      <c r="B44" s="10" t="s">
+      <c r="C44" s="18"/>
+      <c r="D44" s="45"/>
+      <c r="E44" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="15">
+        <v>1000000</v>
+      </c>
+      <c r="G44" s="45"/>
+      <c r="H44" s="15"/>
+    </row>
+    <row r="45" ht="15" spans="1:8">
+      <c r="A45" s="39"/>
+      <c r="B45" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C44" s="34"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F44" s="12">
-        <v>1000000</v>
-      </c>
-      <c r="G44" s="35"/>
-      <c r="H44" s="12"/>
-    </row>
-    <row r="45" ht="16.8" spans="1:8">
-      <c r="A45" s="36"/>
-      <c r="B45" s="10" t="s">
+      <c r="C45" s="18"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="15">
+        <v>3000000</v>
+      </c>
+      <c r="G45" s="45"/>
+      <c r="H45" s="15"/>
+    </row>
+    <row r="46" ht="15" spans="1:8">
+      <c r="A46" s="46"/>
+      <c r="B46" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="34"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F45" s="12">
-        <v>3000000</v>
-      </c>
-      <c r="G45" s="35"/>
-      <c r="H45" s="12"/>
-    </row>
-    <row r="46" ht="16.8" spans="1:8">
-      <c r="A46" s="37"/>
-      <c r="B46" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C46" s="34"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F46" s="12">
+      <c r="C46" s="18"/>
+      <c r="D46" s="45"/>
+      <c r="E46" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="15">
         <v>1800000</v>
       </c>
-      <c r="G46" s="35"/>
-      <c r="H46" s="12"/>
+      <c r="G46" s="45"/>
+      <c r="H46" s="15"/>
     </row>
     <row r="47" spans="6:6">
       <c r="F47" s="4"/>
@@ -2783,7 +2763,7 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F52" s="4"/>
     </row>
@@ -2792,7 +2772,7 @@
         <v>25</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F53" s="4"/>
     </row>

</xml_diff>

<commit_message>
15 jan 2026 17:25 PM
</commit_message>
<xml_diff>
--- a/SUPPLIER RELATED/SUPPLIER PAYMENT STATUS.xlsx
+++ b/SUPPLIER RELATED/SUPPLIER PAYMENT STATUS.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17020"/>
+    <workbookView windowWidth="27080" windowHeight="17020"/>
   </bookViews>
   <sheets>
     <sheet name="SUPPLIER PAYMENT STATUS" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="81">
   <si>
     <t>DIVISION</t>
   </si>
@@ -74,7 +74,7 @@
     <t>PAID 1/2</t>
   </si>
   <si>
-    <t>5 &amp; 25 JAN</t>
+    <t>15 &amp; 25 JAN</t>
   </si>
   <si>
     <t>OUTSTANDING CONFIRMED</t>
@@ -89,21 +89,36 @@
     <t>RAFI SEAFOOD (SEAFOOD)</t>
   </si>
   <si>
+    <t>MAMA RADA PRODUCTION</t>
+  </si>
+  <si>
+    <t>N/O</t>
+  </si>
+  <si>
+    <t>KSP (CHICKEN)</t>
+  </si>
+  <si>
     <t>MAKER</t>
   </si>
   <si>
-    <t>MAMA RADA PRODUCTION</t>
-  </si>
-  <si>
-    <t>N/O</t>
-  </si>
-  <si>
-    <t>KSP (CHICKEN)</t>
-  </si>
-  <si>
     <t>SURYA CIPTA NIAGA (STEAK MEAT)</t>
   </si>
   <si>
+    <r>
+      <t>NOTE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: BU BUNGA Bill's shown on status is only half of the total bill and MulIa Jaya has been removed from the lists since it's paid by petty cash. There's also small revision on BU BUNGA 1st payment due date which is supposed to be 15th instead of 5th of each month.</t>
+    </r>
+  </si>
+  <si>
     <t>BAYU AGNI (LPG GAS)</t>
   </si>
   <si>
@@ -119,7 +134,7 @@
     <t>BOILER (DUMPLINGS)</t>
   </si>
   <si>
-    <t>DISHY SOAP CHEMICALS)</t>
+    <t>DISHY SOAP (CHEMICALS)</t>
   </si>
   <si>
     <t>DAILY BAGUETTE (BREAD)</t>
@@ -134,6 +149,9 @@
     <t>PAID 2ND</t>
   </si>
   <si>
+    <t>PAID 3ND</t>
+  </si>
+  <si>
     <t>BAR</t>
   </si>
   <si>
@@ -149,18 +167,24 @@
     <t>PNB (ALCOHOL)</t>
   </si>
   <si>
-    <t>TOTAL DECEMBER BILL (TENTATIVE)</t>
+    <t>TOTAL DECEMBER'S BILL</t>
   </si>
   <si>
     <t>DSP (ALCOHOL)</t>
   </si>
   <si>
+    <t>INITIAL</t>
+  </si>
+  <si>
     <t>DSP ARYA BIMA (ALCOHOL)</t>
   </si>
   <si>
     <t>SELERA (STIR UP SYRUP)</t>
   </si>
   <si>
+    <t>UNPAID</t>
+  </si>
+  <si>
     <t>DW BALI (ALCOHOL)</t>
   </si>
   <si>
@@ -185,12 +209,6 @@
     <t>CHAI CHITAI (TEA)</t>
   </si>
   <si>
-    <t>MULIA JAYA (PASSION FRUIT)</t>
-  </si>
-  <si>
-    <t>BY CASH</t>
-  </si>
-  <si>
     <t>DEWATA KENCANA DISTRIBUSI (ICELAND)</t>
   </si>
   <si>
@@ -230,13 +248,7 @@
     <t>COFFEE MACHINE MAINTENANCE</t>
   </si>
   <si>
-    <t>cling</t>
-  </si>
-  <si>
     <t>TWIN PACK MINI &amp; ANT KILLER (TKP)</t>
-  </si>
-  <si>
-    <t>plastic vacuum</t>
   </si>
   <si>
     <t>GLASS TISSUE BOX (TKP)</t>
@@ -276,7 +288,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -284,6 +296,7 @@
     <numFmt numFmtId="180" formatCode="[$-409]d\-mmm\-yyyy;@"/>
     <numFmt numFmtId="181" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="182" formatCode="[$-809]dd\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="183" formatCode="[$Rp-421]#,##0.00;[Red][$Rp-421]#,##0.00"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -461,7 +474,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -518,6 +531,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -703,7 +728,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -1025,6 +1050,37 @@
         <color auto="1"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1151,7 +1207,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="28" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1163,119 +1219,119 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="28" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="29" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="28" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="32" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="33" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="35" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1408,9 +1464,6 @@
     <xf numFmtId="180" fontId="2" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1504,7 +1557,40 @@
     <xf numFmtId="181" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
@@ -2043,7 +2129,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="17.6"/>
   <cols>
     <col min="1" max="1" width="18.4375" style="2" customWidth="1"/>
@@ -2056,9 +2142,11 @@
     <col min="9" max="9" width="14.3359375" style="4"/>
     <col min="10" max="10" width="17.7109375" customWidth="1"/>
     <col min="11" max="11" width="17.3125" style="6"/>
-    <col min="12" max="12" width="22.6640625" style="4" customWidth="1"/>
-    <col min="13" max="13" width="15.25"/>
-    <col min="14" max="14" width="19.140625" customWidth="1"/>
+    <col min="12" max="12" width="26.125" style="4" customWidth="1"/>
+    <col min="13" max="13" width="5.8671875" customWidth="1"/>
+    <col min="14" max="14" width="16.9375" customWidth="1"/>
+    <col min="15" max="15" width="7.9375" customWidth="1"/>
+    <col min="17" max="17" width="15.25"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.35" spans="1:12">
@@ -2074,32 +2162,32 @@
       <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="E1" s="46" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="G1" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="49" t="s">
+      <c r="H1" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="48" t="s">
+      <c r="I1" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="57" t="s">
+      <c r="J1" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="58" t="s">
+      <c r="K1" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="59" t="s">
+      <c r="L1" s="58" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" ht="16.8" spans="1:12">
       <c r="A2" s="11" t="s">
         <v>9</v>
       </c>
@@ -2118,26 +2206,26 @@
       <c r="F2" s="14">
         <v>39738000</v>
       </c>
-      <c r="G2" s="50" t="s">
+      <c r="G2" s="49" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="18">
         <v>34233500</v>
       </c>
-      <c r="I2" s="50" t="s">
+      <c r="I2" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="60">
+      <c r="J2" s="59">
         <v>42310500</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="61" t="s">
+      <c r="L2" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" ht="16.8" spans="1:12">
       <c r="A3" s="15"/>
       <c r="B3" s="16" t="s">
         <v>17</v>
@@ -2163,17 +2251,17 @@
       <c r="I3" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="62">
+      <c r="J3" s="61">
         <v>48169400</v>
       </c>
       <c r="K3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L3" s="61" t="s">
+      <c r="L3" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" ht="16.8" spans="1:12">
       <c r="A4" s="15"/>
       <c r="B4" s="16" t="s">
         <v>19</v>
@@ -2196,23 +2284,23 @@
       <c r="H4" s="18">
         <v>21943450</v>
       </c>
-      <c r="I4" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="62">
+      <c r="I4" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="61">
         <v>36138000</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="61" t="s">
+      <c r="L4" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" ht="16.8" spans="1:10">
       <c r="A5" s="15"/>
       <c r="B5" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>11</v>
@@ -2233,14 +2321,14 @@
         <v>320000</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="62"/>
+        <v>21</v>
+      </c>
+      <c r="J5" s="61"/>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="15"/>
       <c r="B6" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>11</v>
@@ -2261,16 +2349,16 @@
         <v>5069850</v>
       </c>
       <c r="I6" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="62">
+        <v>23</v>
+      </c>
+      <c r="J6" s="61">
         <v>6026050</v>
       </c>
-      <c r="L6" s="61" t="s">
+      <c r="L6" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:15">
       <c r="A7" s="15"/>
       <c r="B7" s="16" t="s">
         <v>24</v>
@@ -2293,23 +2381,27 @@
       <c r="H7" s="18">
         <v>13417600</v>
       </c>
-      <c r="I7" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="62">
+      <c r="I7" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="61">
         <v>9006800</v>
       </c>
       <c r="K7" s="6">
         <v>46027</v>
       </c>
-      <c r="L7" s="61" t="s">
+      <c r="L7" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:12">
+      <c r="N7" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="O7" s="76"/>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="15"/>
       <c r="B8" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>11</v>
@@ -2330,77 +2422,83 @@
         <v>5850000</v>
       </c>
       <c r="I8" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="62">
+        <v>23</v>
+      </c>
+      <c r="J8" s="61">
         <v>8775000</v>
       </c>
       <c r="K8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="61" t="s">
+      <c r="L8" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="N8" s="77"/>
+      <c r="O8" s="78"/>
+    </row>
+    <row r="9" ht="16.8" spans="1:15">
       <c r="A9" s="15"/>
       <c r="B9" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="18"/>
       <c r="E9" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F9" s="18"/>
       <c r="G9" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H9" s="18"/>
       <c r="I9" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="62"/>
-    </row>
-    <row r="10" spans="1:12">
+        <v>21</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="N9" s="77"/>
+      <c r="O9" s="78"/>
+    </row>
+    <row r="10" ht="16.8" spans="1:15">
       <c r="A10" s="15"/>
       <c r="B10" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="18"/>
       <c r="E10" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F10" s="18"/>
       <c r="G10" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H10" s="18"/>
       <c r="I10" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="62">
+      <c r="J10" s="61">
         <v>160000</v>
       </c>
       <c r="K10" s="6">
-        <v>46021</v>
-      </c>
-      <c r="L10" s="61" t="s">
+        <v>46386</v>
+      </c>
+      <c r="L10" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:12">
+      <c r="N10" s="77"/>
+      <c r="O10" s="78"/>
+    </row>
+    <row r="11" ht="16.8" spans="1:15">
       <c r="A11" s="15"/>
       <c r="B11" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" s="18"/>
       <c r="E11" s="17" t="s">
@@ -2415,23 +2513,25 @@
       <c r="H11" s="18">
         <v>152000</v>
       </c>
-      <c r="I11" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="62">
+      <c r="I11" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="61">
         <v>329000</v>
       </c>
       <c r="K11" s="6">
-        <v>46017</v>
-      </c>
-      <c r="L11" s="61" t="s">
+        <v>46382</v>
+      </c>
+      <c r="L11" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:12">
+      <c r="N11" s="77"/>
+      <c r="O11" s="78"/>
+    </row>
+    <row r="12" ht="16.8" spans="1:15">
       <c r="A12" s="15"/>
       <c r="B12" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>11</v>
@@ -2452,20 +2552,22 @@
       <c r="I12" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J12" s="62">
+      <c r="J12" s="61">
         <v>319000</v>
       </c>
       <c r="K12" s="6">
-        <v>46015</v>
-      </c>
-      <c r="L12" s="61" t="s">
+        <v>46380</v>
+      </c>
+      <c r="L12" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="13" spans="1:12">
+      <c r="N12" s="77"/>
+      <c r="O12" s="78"/>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="15"/>
       <c r="B13" s="16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>11</v>
@@ -2483,19 +2585,21 @@
       <c r="H13" s="18">
         <v>995000</v>
       </c>
-      <c r="I13" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" s="62">
+      <c r="I13" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="61">
         <v>2855000</v>
       </c>
-      <c r="K13" s="63"/>
-      <c r="L13" s="64"/>
-    </row>
-    <row r="14" spans="1:12">
+      <c r="K13" s="62"/>
+      <c r="L13" s="63"/>
+      <c r="N13" s="77"/>
+      <c r="O13" s="78"/>
+    </row>
+    <row r="14" ht="16.8" spans="1:15">
       <c r="A14" s="15"/>
       <c r="B14" s="16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>11</v>
@@ -2513,49 +2617,53 @@
       <c r="H14" s="18">
         <v>2996000</v>
       </c>
-      <c r="I14" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" s="62">
+      <c r="I14" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="J14" s="61">
         <v>1044000</v>
       </c>
-      <c r="K14" s="63"/>
-      <c r="L14" s="64"/>
-    </row>
-    <row r="15" spans="1:12">
+      <c r="K14" s="62"/>
+      <c r="L14" s="63"/>
+      <c r="N14" s="77"/>
+      <c r="O14" s="78"/>
+    </row>
+    <row r="15" ht="17.55" spans="1:15">
       <c r="A15" s="20"/>
       <c r="B15" s="21" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C15" s="22"/>
       <c r="D15" s="23"/>
-      <c r="E15" s="51" t="s">
-        <v>33</v>
+      <c r="E15" s="50" t="s">
+        <v>34</v>
       </c>
       <c r="F15" s="23">
         <v>10000000</v>
       </c>
-      <c r="G15" s="51" t="s">
-        <v>34</v>
+      <c r="G15" s="50" t="s">
+        <v>35</v>
       </c>
       <c r="H15" s="18">
         <v>10000000</v>
       </c>
-      <c r="I15" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J15" s="65">
+      <c r="I15" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15" s="64">
         <v>10000000</v>
       </c>
-      <c r="K15" s="66"/>
-      <c r="L15" s="67"/>
-    </row>
-    <row r="16" spans="1:12">
+      <c r="K15" s="65"/>
+      <c r="L15" s="66"/>
+      <c r="N15" s="77"/>
+      <c r="O15" s="78"/>
+    </row>
+    <row r="16" ht="17.55" spans="1:15">
       <c r="A16" s="24" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>11</v>
@@ -2576,22 +2684,24 @@
         <v>12478500</v>
       </c>
       <c r="I16" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J16" s="60">
+        <v>23</v>
+      </c>
+      <c r="J16" s="59">
         <v>14051500</v>
       </c>
-      <c r="K16" s="66" t="s">
+      <c r="K16" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="L16" s="68" t="s">
+      <c r="L16" s="67" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:12">
+      <c r="N16" s="79"/>
+      <c r="O16" s="80"/>
+    </row>
+    <row r="17" ht="16.8" spans="1:12">
       <c r="A17" s="25"/>
       <c r="B17" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>11</v>
@@ -2611,23 +2721,23 @@
       <c r="H17" s="18">
         <v>1800000</v>
       </c>
-      <c r="I17" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J17" s="62">
+      <c r="I17" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J17" s="61">
         <v>2860000</v>
       </c>
-      <c r="K17" s="66" t="s">
+      <c r="K17" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="L17" s="69" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
+      <c r="L17" s="68" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" ht="16.8" spans="1:15">
       <c r="A18" s="25"/>
       <c r="B18" s="16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>11</v>
@@ -2647,26 +2757,27 @@
       <c r="H18" s="18">
         <v>7025000</v>
       </c>
-      <c r="I18" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J18" s="62">
+      <c r="I18" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J18" s="61">
         <v>4175000</v>
       </c>
       <c r="K18" s="6">
         <v>46052</v>
       </c>
-      <c r="L18" s="68" t="s">
+      <c r="L18" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="N18" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
+      <c r="N18" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="O18" s="81"/>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" s="25"/>
       <c r="B19" s="16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>11</v>
@@ -2687,56 +2798,66 @@
         <v>12023500</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J19" s="62">
+        <v>23</v>
+      </c>
+      <c r="J19" s="61">
         <v>18173500</v>
       </c>
       <c r="K19" s="6">
         <v>46051</v>
       </c>
-      <c r="L19" s="68" t="s">
+      <c r="L19" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="N19" s="76">
+      <c r="N19" s="82">
         <f>SUM(J2:J50)+42310500</f>
-        <v>312314366</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <v>312960866</v>
+      </c>
+      <c r="O19" s="42" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" ht="16.8" spans="1:15">
       <c r="A20" s="25"/>
       <c r="B20" s="16" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" s="18"/>
       <c r="E20" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F20" s="18"/>
       <c r="G20" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H20" s="18"/>
-      <c r="I20" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J20" s="62">
+      <c r="I20" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J20" s="61">
         <v>3633750</v>
       </c>
       <c r="K20" s="6">
         <v>46035</v>
       </c>
-      <c r="L20" s="61" t="s">
+      <c r="L20" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="21" spans="1:14">
+      <c r="N20" s="82">
+        <f>SUMIFS(J2:J50,I2:I50,"*PAID*")</f>
+        <v>211559316</v>
+      </c>
+      <c r="O20" s="83" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" ht="16.8" spans="1:17">
       <c r="A21" s="25"/>
       <c r="B21" s="16" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>11</v>
@@ -2756,24 +2877,31 @@
       <c r="H21" s="18">
         <v>1665000</v>
       </c>
-      <c r="I21" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" s="62">
+      <c r="I21" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J21" s="61">
         <v>3552000</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L21" s="61" t="s">
+      <c r="L21" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="N21" s="77"/>
-    </row>
-    <row r="22" spans="1:12">
+      <c r="N21" s="84">
+        <f>N19-N20</f>
+        <v>101401550</v>
+      </c>
+      <c r="O21" s="85" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q21" s="87"/>
+    </row>
+    <row r="22" ht="16.8" spans="1:17">
       <c r="A22" s="25"/>
       <c r="B22" s="16" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>11</v>
@@ -2782,7 +2910,7 @@
         <v>2410000</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F22" s="18"/>
       <c r="G22" s="17" t="s">
@@ -2792,22 +2920,24 @@
         <v>2110000</v>
       </c>
       <c r="I22" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J22" s="62">
+        <v>23</v>
+      </c>
+      <c r="J22" s="61">
         <v>12065000</v>
       </c>
       <c r="K22" s="6">
         <v>46036</v>
       </c>
-      <c r="L22" s="61" t="s">
+      <c r="L22" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="1:12">
+      <c r="N22" s="86"/>
+      <c r="Q22" s="87"/>
+    </row>
+    <row r="23" ht="16.8" spans="1:14">
       <c r="A23" s="25"/>
       <c r="B23" s="16" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>11</v>
@@ -2827,26 +2957,27 @@
       <c r="H23" s="18">
         <v>1750003</v>
       </c>
-      <c r="I23" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J23" s="62">
+      <c r="I23" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="61">
         <v>1837503</v>
       </c>
       <c r="K23" s="6">
         <v>46036</v>
       </c>
-      <c r="L23" s="61" t="s">
+      <c r="L23" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:10">
+      <c r="N23" s="87"/>
+    </row>
+    <row r="24" ht="16.8" spans="1:10">
       <c r="A24" s="25"/>
       <c r="B24" s="16" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D24" s="18"/>
       <c r="E24" s="17" t="s">
@@ -2856,18 +2987,18 @@
         <v>2280000</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H24" s="18"/>
       <c r="I24" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J24" s="62"/>
-    </row>
-    <row r="25" spans="1:12">
+        <v>21</v>
+      </c>
+      <c r="J24" s="61"/>
+    </row>
+    <row r="25" ht="16.8" spans="1:14">
       <c r="A25" s="25"/>
       <c r="B25" s="16" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>11</v>
@@ -2887,23 +3018,24 @@
       <c r="H25" s="18">
         <v>1190009</v>
       </c>
-      <c r="I25" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J25" s="62">
+      <c r="I25" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J25" s="61">
         <v>2380013</v>
       </c>
       <c r="K25" s="6">
         <v>46044</v>
       </c>
-      <c r="L25" s="61" t="s">
+      <c r="L25" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:12">
+      <c r="N25" s="87"/>
+    </row>
+    <row r="26" ht="16.8" spans="1:14">
       <c r="A26" s="25"/>
       <c r="B26" s="16" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>11</v>
@@ -2926,20 +3058,21 @@
       <c r="I26" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J26" s="62">
+      <c r="J26" s="61">
         <v>5600000</v>
       </c>
       <c r="K26" s="6">
         <v>46023</v>
       </c>
-      <c r="L26" s="61" t="s">
+      <c r="L26" s="60" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="27" spans="1:12">
+      <c r="N26" s="87"/>
+    </row>
+    <row r="27" ht="16.8" spans="1:12">
       <c r="A27" s="25"/>
       <c r="B27" s="16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C27" s="17" t="s">
         <v>11</v>
@@ -2959,45 +3092,45 @@
       <c r="H27" s="18">
         <v>600000</v>
       </c>
-      <c r="I27" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J27" s="62">
+      <c r="I27" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J27" s="61">
         <v>915750</v>
       </c>
       <c r="K27" s="6">
-        <v>46013</v>
-      </c>
-      <c r="L27" s="61" t="s">
+        <v>46378</v>
+      </c>
+      <c r="L27" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" ht="16.8" spans="1:10">
       <c r="A28" s="25"/>
       <c r="B28" s="16" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D28" s="18"/>
       <c r="E28" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F28" s="18"/>
       <c r="G28" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H28" s="18"/>
       <c r="I28" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28" s="62"/>
-    </row>
-    <row r="29" spans="1:10">
+        <v>21</v>
+      </c>
+      <c r="J28" s="61"/>
+    </row>
+    <row r="29" ht="16.8" spans="1:10">
       <c r="A29" s="25"/>
       <c r="B29" s="16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>11</v>
@@ -3006,306 +3139,302 @@
         <v>3948000</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F29" s="18"/>
       <c r="G29" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H29" s="18"/>
       <c r="I29" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="62"/>
-    </row>
-    <row r="30" spans="1:10">
+        <v>21</v>
+      </c>
+      <c r="J29" s="61"/>
+    </row>
+    <row r="30" ht="16.8" spans="1:12">
       <c r="A30" s="25"/>
       <c r="B30" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D30" s="18">
-        <v>250000</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C30" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" s="18"/>
       <c r="E30" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="F30" s="18">
-        <v>300000</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F30" s="18"/>
       <c r="G30" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="H30" s="18">
-        <v>300000</v>
-      </c>
-      <c r="I30" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="J30" s="62">
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
+        <v>21</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J30" s="61">
+        <v>975300</v>
+      </c>
+      <c r="K30" s="6">
+        <v>46031</v>
+      </c>
+      <c r="L30" s="60" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" ht="16.8" spans="1:12">
       <c r="A31" s="25"/>
       <c r="B31" s="16" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D31" s="18"/>
       <c r="E31" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F31" s="18"/>
       <c r="G31" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H31" s="18"/>
       <c r="I31" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="J31" s="62">
-        <v>975300</v>
+      <c r="J31" s="61">
+        <v>1600000</v>
       </c>
       <c r="K31" s="6">
-        <v>46031</v>
-      </c>
-      <c r="L31" s="61" t="s">
+        <v>46383</v>
+      </c>
+      <c r="L31" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" ht="16.8" spans="1:10">
       <c r="A32" s="25"/>
       <c r="B32" s="16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D32" s="18"/>
-      <c r="E32" s="19" t="s">
-        <v>22</v>
+      <c r="E32" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="F32" s="18"/>
-      <c r="G32" s="19" t="s">
-        <v>22</v>
+      <c r="G32" s="26" t="s">
+        <v>21</v>
       </c>
       <c r="H32" s="18"/>
-      <c r="I32" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="J32" s="62">
-        <v>1600000</v>
-      </c>
-      <c r="K32" s="6">
-        <v>46018</v>
-      </c>
-      <c r="L32" s="61" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10">
-      <c r="A33" s="25"/>
-      <c r="B33" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="F33" s="18"/>
-      <c r="G33" s="26" t="s">
-        <v>22</v>
+      <c r="I32" s="39"/>
+      <c r="J32" s="61"/>
+    </row>
+    <row r="33" ht="17.55" spans="1:10">
+      <c r="A33" s="27"/>
+      <c r="B33" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="30"/>
+      <c r="E33" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="30">
+        <v>915750</v>
+      </c>
+      <c r="G33" s="51" t="s">
+        <v>21</v>
       </c>
       <c r="H33" s="18"/>
       <c r="I33" s="39"/>
-      <c r="J33" s="62"/>
-    </row>
-    <row r="34" spans="1:10">
-      <c r="A34" s="27"/>
-      <c r="B34" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="30">
-        <v>915750</v>
-      </c>
-      <c r="G34" s="52" t="s">
-        <v>22</v>
-      </c>
-      <c r="H34" s="18"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="70"/>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="14">
+      <c r="J33" s="69"/>
+    </row>
+    <row r="34" ht="17.55" spans="1:12">
+      <c r="A34" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="14">
         <v>4897000</v>
       </c>
+      <c r="E34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="14">
+        <v>8368100</v>
+      </c>
+      <c r="G34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" s="18">
+        <v>4047600</v>
+      </c>
+      <c r="I34" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J34" s="59">
+        <v>1897000</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L34" s="60" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" ht="16.8" spans="1:10">
+      <c r="A35" s="15"/>
+      <c r="B35" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="18">
+        <v>4375000</v>
+      </c>
       <c r="E35" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F35" s="14">
-        <v>8368100</v>
-      </c>
-      <c r="G35" s="13" t="s">
+      <c r="F35" s="18">
+        <v>4715000</v>
+      </c>
+      <c r="G35" s="17" t="s">
         <v>11</v>
       </c>
       <c r="H35" s="18">
-        <v>4047600</v>
-      </c>
-      <c r="I35" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J35" s="60">
-        <v>1897000</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="L35" s="61" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10">
+        <v>2585000</v>
+      </c>
+      <c r="I35" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J35" s="61">
+        <v>27100000</v>
+      </c>
+    </row>
+    <row r="36" ht="16.8" spans="1:10">
       <c r="A36" s="15"/>
       <c r="B36" s="16" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C36" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D36" s="18">
-        <v>4375000</v>
-      </c>
-      <c r="E36" s="13" t="s">
+        <v>1007480.64</v>
+      </c>
+      <c r="E36" s="17" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="18">
-        <v>4715000</v>
-      </c>
-      <c r="G36" s="17" t="s">
+        <v>638483</v>
+      </c>
+      <c r="G36" s="33" t="s">
         <v>11</v>
       </c>
       <c r="H36" s="18">
-        <v>2585000</v>
-      </c>
-      <c r="I36" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="J36" s="62">
-        <v>27100000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
-      <c r="A37" s="15"/>
-      <c r="B37" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="18">
-        <v>1007480.64</v>
-      </c>
-      <c r="E37" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="18">
-        <v>638483</v>
+        <v>269482</v>
+      </c>
+      <c r="I36" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="J36" s="61"/>
+    </row>
+    <row r="37" ht="17.55" spans="1:12">
+      <c r="A37" s="31"/>
+      <c r="B37" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="34">
+        <v>1168000</v>
+      </c>
+      <c r="E37" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="34">
+        <v>893000</v>
       </c>
       <c r="G37" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="H37" s="18">
-        <v>269482</v>
-      </c>
-      <c r="I37" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="J37" s="62"/>
-    </row>
-    <row r="38" spans="1:12">
-      <c r="A38" s="31"/>
-      <c r="B38" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="C38" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="34">
-        <v>1168000</v>
-      </c>
-      <c r="E38" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="34">
-        <v>893000</v>
-      </c>
-      <c r="G38" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="H38" s="34">
+      <c r="H37" s="34">
         <v>847000</v>
       </c>
-      <c r="I38" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="J38" s="71">
+      <c r="I37" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="J37" s="70">
         <v>944000</v>
       </c>
-      <c r="K38" s="6">
+      <c r="K37" s="6">
         <v>46027</v>
       </c>
-      <c r="L38" s="61" t="s">
+      <c r="L37" s="60" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
-      <c r="A39" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="36"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="14">
+    <row r="38" ht="16.8" spans="1:10">
+      <c r="A38" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="36"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="14">
         <v>1020000</v>
       </c>
-      <c r="G39" s="37"/>
-      <c r="H39" s="53"/>
-      <c r="I39" s="72"/>
-      <c r="J39" s="73"/>
-    </row>
-    <row r="40" spans="1:10">
+      <c r="G38" s="37"/>
+      <c r="H38" s="52"/>
+      <c r="I38" s="71"/>
+      <c r="J38" s="72"/>
+    </row>
+    <row r="39" ht="16.8" spans="1:10">
+      <c r="A39" s="38"/>
+      <c r="B39" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C39" s="39"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="18">
+        <v>1350000</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H39" s="53">
+        <v>1800000</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="J39" s="73">
+        <v>1850000</v>
+      </c>
+    </row>
+    <row r="40" ht="16.8" spans="1:10">
       <c r="A40" s="38"/>
       <c r="B40" s="16" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C40" s="39"/>
       <c r="D40" s="40"/>
@@ -3313,25 +3442,17 @@
         <v>11</v>
       </c>
       <c r="F40" s="18">
-        <v>1350000</v>
-      </c>
-      <c r="G40" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="H40" s="54">
-        <v>1800000</v>
-      </c>
-      <c r="I40" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="J40" s="74">
-        <v>1850000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12">
+        <v>600000</v>
+      </c>
+      <c r="G40" s="40"/>
+      <c r="H40" s="53"/>
+      <c r="I40" s="41"/>
+      <c r="J40" s="73"/>
+    </row>
+    <row r="41" ht="16.8" spans="1:10">
       <c r="A41" s="38"/>
       <c r="B41" s="16" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C41" s="39"/>
       <c r="D41" s="40"/>
@@ -3339,20 +3460,17 @@
         <v>11</v>
       </c>
       <c r="F41" s="18">
-        <v>600000</v>
+        <v>318134</v>
       </c>
       <c r="G41" s="40"/>
-      <c r="H41" s="54"/>
+      <c r="H41" s="53"/>
       <c r="I41" s="41"/>
-      <c r="J41" s="74"/>
-      <c r="L41" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12">
+      <c r="J41" s="73"/>
+    </row>
+    <row r="42" ht="16.8" spans="1:10">
       <c r="A42" s="38"/>
       <c r="B42" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C42" s="39"/>
       <c r="D42" s="40"/>
@@ -3360,20 +3478,17 @@
         <v>11</v>
       </c>
       <c r="F42" s="18">
-        <v>318134</v>
+        <v>248700</v>
       </c>
       <c r="G42" s="40"/>
-      <c r="H42" s="54"/>
+      <c r="H42" s="53"/>
       <c r="I42" s="41"/>
-      <c r="J42" s="74"/>
-      <c r="L42" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10">
+      <c r="J42" s="73"/>
+    </row>
+    <row r="43" ht="16.8" spans="1:10">
       <c r="A43" s="38"/>
       <c r="B43" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C43" s="39"/>
       <c r="D43" s="40"/>
@@ -3381,17 +3496,17 @@
         <v>11</v>
       </c>
       <c r="F43" s="18">
-        <v>248700</v>
+        <v>1029180</v>
       </c>
       <c r="G43" s="40"/>
-      <c r="H43" s="54"/>
+      <c r="H43" s="53"/>
       <c r="I43" s="41"/>
-      <c r="J43" s="74"/>
-    </row>
-    <row r="44" spans="1:10">
+      <c r="J43" s="73"/>
+    </row>
+    <row r="44" ht="16.8" spans="1:10">
       <c r="A44" s="38"/>
       <c r="B44" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C44" s="39"/>
       <c r="D44" s="40"/>
@@ -3399,17 +3514,17 @@
         <v>11</v>
       </c>
       <c r="F44" s="18">
-        <v>1029180</v>
+        <v>270000</v>
       </c>
       <c r="G44" s="40"/>
-      <c r="H44" s="54"/>
+      <c r="H44" s="53"/>
       <c r="I44" s="41"/>
-      <c r="J44" s="74"/>
-    </row>
-    <row r="45" spans="1:10">
+      <c r="J44" s="73"/>
+    </row>
+    <row r="45" ht="16.8" spans="1:10">
       <c r="A45" s="38"/>
       <c r="B45" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C45" s="39"/>
       <c r="D45" s="40"/>
@@ -3417,17 +3532,17 @@
         <v>11</v>
       </c>
       <c r="F45" s="18">
-        <v>270000</v>
+        <v>1000000</v>
       </c>
       <c r="G45" s="40"/>
-      <c r="H45" s="54"/>
+      <c r="H45" s="53"/>
       <c r="I45" s="41"/>
-      <c r="J45" s="74"/>
-    </row>
-    <row r="46" spans="1:10">
+      <c r="J45" s="73"/>
+    </row>
+    <row r="46" ht="16.8" spans="1:10">
       <c r="A46" s="38"/>
       <c r="B46" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C46" s="39"/>
       <c r="D46" s="40"/>
@@ -3435,17 +3550,17 @@
         <v>11</v>
       </c>
       <c r="F46" s="18">
-        <v>1000000</v>
+        <v>3000000</v>
       </c>
       <c r="G46" s="40"/>
-      <c r="H46" s="54"/>
+      <c r="H46" s="53"/>
       <c r="I46" s="41"/>
-      <c r="J46" s="74"/>
-    </row>
-    <row r="47" spans="1:10">
+      <c r="J46" s="73"/>
+    </row>
+    <row r="47" ht="16.8" spans="1:10">
       <c r="A47" s="38"/>
       <c r="B47" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C47" s="39"/>
       <c r="D47" s="40"/>
@@ -3453,112 +3568,96 @@
         <v>11</v>
       </c>
       <c r="F47" s="18">
-        <v>3000000</v>
+        <v>1800000</v>
       </c>
       <c r="G47" s="40"/>
-      <c r="H47" s="54"/>
+      <c r="H47" s="53"/>
       <c r="I47" s="41"/>
-      <c r="J47" s="74"/>
-    </row>
-    <row r="48" spans="1:10">
+      <c r="J47" s="73"/>
+    </row>
+    <row r="48" ht="16.8" spans="1:10">
       <c r="A48" s="38"/>
       <c r="B48" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="40"/>
-      <c r="E48" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48" s="18">
-        <v>1800000</v>
-      </c>
-      <c r="G48" s="40"/>
-      <c r="H48" s="54"/>
+        <v>76</v>
+      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="42"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="54">
+        <v>2450000</v>
+      </c>
       <c r="I48" s="41"/>
-      <c r="J48" s="74"/>
-    </row>
-    <row r="49" spans="1:10">
+      <c r="J48" s="73"/>
+    </row>
+    <row r="49" ht="16.8" spans="1:10">
       <c r="A49" s="38"/>
       <c r="B49" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C49" s="41"/>
       <c r="D49" s="42"/>
       <c r="E49" s="41"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="H49" s="55">
-        <v>2450000</v>
-      </c>
-      <c r="I49" s="41"/>
-      <c r="J49" s="74"/>
-    </row>
-    <row r="50" spans="1:10">
-      <c r="A50" s="38"/>
-      <c r="B50" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C50" s="41"/>
-      <c r="D50" s="42"/>
-      <c r="E50" s="41"/>
+      <c r="F49" s="54"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="54"/>
+      <c r="I49" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="J49" s="73">
+        <v>860800</v>
+      </c>
+    </row>
+    <row r="50" ht="17.55" spans="1:10">
+      <c r="A50" s="43"/>
+      <c r="B50" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="44"/>
+      <c r="D50" s="45"/>
+      <c r="E50" s="44"/>
       <c r="F50" s="55"/>
-      <c r="G50" s="42"/>
+      <c r="G50" s="45"/>
       <c r="H50" s="55"/>
       <c r="I50" s="17" t="s">
         <v>11</v>
       </c>
       <c r="J50" s="74">
-        <v>860800</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="43"/>
-      <c r="B51" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="C51" s="45"/>
-      <c r="D51" s="46"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="46"/>
-      <c r="H51" s="56"/>
-      <c r="I51" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="J51" s="75">
         <v>1046500</v>
       </c>
+    </row>
+    <row r="51" spans="6:6">
+      <c r="F51" s="5"/>
     </row>
     <row r="52" spans="6:6">
       <c r="F52" s="5"/>
     </row>
-    <row r="53" spans="6:6">
+    <row r="53" spans="1:6">
+      <c r="A53" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="F53" s="5"/>
     </row>
-    <row r="54" spans="1:6">
-      <c r="A54" s="2" t="s">
-        <v>79</v>
+    <row r="54" ht="16.8" spans="1:6">
+      <c r="A54" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>80</v>
       </c>
       <c r="F54" s="5"/>
     </row>
-    <row r="55" spans="1:6">
-      <c r="A55" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F55" s="5"/>
-    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="N18:O18"/>
     <mergeCell ref="A2:A15"/>
-    <mergeCell ref="A16:A34"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="A39:A51"/>
+    <mergeCell ref="A16:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A50"/>
+    <mergeCell ref="N7:O16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>